<commit_message>
Arquivos finais de documentação
</commit_message>
<xml_diff>
--- a/4.Teste/CONIM - Roteiro de Teste.xlsx
+++ b/4.Teste/CONIM - Roteiro de Teste.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rosag\Documents\CONIM_ContractImovel\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C54D2A-C38B-4AC0-9A51-F69F97FC94F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53719EA-3A87-40F5-81D8-4F6852C70AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="913" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="110">
   <si>
     <t>Caso de Uso</t>
   </si>
@@ -155,9 +155,6 @@
     <t>Buscar imóvel inexistente</t>
   </si>
   <si>
-    <t>Erro ao associar inquilino ao imóvel</t>
-  </si>
-  <si>
     <t>Endereço = “Rua das Laranjeiras, 12”</t>
   </si>
   <si>
@@ -165,9 +162,6 @@
   </si>
   <si>
     <t>Mostra imóvel “Av. Brasil, 202”</t>
-  </si>
-  <si>
-    <t>Exibe associação incorreta de inquilino</t>
   </si>
   <si>
     <t>Exibe informações completas 
@@ -195,9 +189,6 @@
     <t>CSNF001</t>
   </si>
   <si>
-    <t>Acesso e gerenciamente de usuários</t>
-  </si>
-  <si>
     <t>Alterar status do imóvel</t>
   </si>
   <si>
@@ -217,12 +208,6 @@
   </si>
   <si>
     <t>Ao ter apenas 1 imóvel cadastrado é mostrado ele ao consultar um inexistente.</t>
-  </si>
-  <si>
-    <t>Imóvel Status = 'Em Reforma'</t>
-  </si>
-  <si>
-    <t>O imovél não é mostrado para alocar um novo contrato</t>
   </si>
   <si>
     <t>Erro ao incluir CPF invalido</t>
@@ -348,6 +333,52 @@
   </si>
   <si>
     <t>Imovéis com status diferentes de disponiveis, estão sendo mostrados.</t>
+  </si>
+  <si>
+    <t>Tabela atualiza ao salvar um novo imóvel</t>
+  </si>
+  <si>
+    <t>Cadastrar novo imóvel</t>
+  </si>
+  <si>
+    <t>Tabela é atualizada sem necessidade de atualizar a página</t>
+  </si>
+  <si>
+    <t>A tabela de imóveis não é atuliazada ao cadastrar um novo</t>
+  </si>
+  <si>
+    <t>Gerenciar usuários</t>
+  </si>
+  <si>
+    <t>Visualizar usuário do sistema existente</t>
+  </si>
+  <si>
+    <t>usuario ID = 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exibe corretamente os dados do 
+usuario </t>
+  </si>
+  <si>
+    <t>Salvar sem Campos obrigatórios</t>
+  </si>
+  <si>
+    <t>Nome = Nulo || Usuário = Nulo || Senha = Nulo|| CPF = Nulo</t>
+  </si>
+  <si>
+    <t>Salvar e após alterar o cargo/permissão</t>
+  </si>
+  <si>
+    <t>Cargo = Adminstrador e logo após Cargo = Corretor</t>
+  </si>
+  <si>
+    <t>A alteração deve ser bem sucedidade a alterar a visualização do usuário ao acessar o sistema</t>
+  </si>
+  <si>
+    <t>Sistema deve retornar tratativa de erro para todos os nulos de campos obrigatórios.</t>
+  </si>
+  <si>
+    <t>A edição reflete dentro da visualização, porém no banco e ao atualizar à mudança não é visualizada</t>
   </si>
 </sst>
 </file>
@@ -1643,9 +1674,7 @@
       <c r="D5" s="22">
         <v>5</v>
       </c>
-      <c r="F5" s="20">
-        <v>0</v>
-      </c>
+      <c r="F5" s="20"/>
       <c r="G5" s="20">
         <v>3</v>
       </c>
@@ -1660,9 +1689,7 @@
       <c r="D6" s="22">
         <v>4</v>
       </c>
-      <c r="F6" s="20">
-        <v>0</v>
-      </c>
+      <c r="F6" s="20"/>
       <c r="G6" s="20">
         <v>3</v>
       </c>
@@ -1680,9 +1707,7 @@
       <c r="F7" s="20">
         <v>1</v>
       </c>
-      <c r="G7" s="20">
-        <v>0</v>
-      </c>
+      <c r="G7" s="20"/>
       <c r="H7" s="20">
         <v>3</v>
       </c>
@@ -1696,9 +1721,7 @@
       <c r="D8" s="22">
         <v>5</v>
       </c>
-      <c r="F8" s="20">
-        <v>0</v>
-      </c>
+      <c r="F8" s="20"/>
       <c r="G8" s="20">
         <v>1</v>
       </c>
@@ -1710,11 +1733,15 @@
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="25"/>
       <c r="C9" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="22"/>
+        <v>46</v>
+      </c>
+      <c r="D9" s="22">
+        <v>3</v>
+      </c>
       <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
+      <c r="G9" s="20">
+        <v>1</v>
+      </c>
       <c r="H9" s="20"/>
       <c r="L9" s="26"/>
     </row>
@@ -1827,7 +1854,7 @@
       </c>
       <c r="D21" s="22">
         <f>SUM(D5:D19)</f>
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F21" s="3">
         <f>SUM(F5:F19)</f>
@@ -1835,7 +1862,7 @@
       </c>
       <c r="G21" s="3">
         <f>SUM(G5:G19)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H21" s="3">
         <f>SUM(H5:H19)</f>
@@ -1843,7 +1870,7 @@
       </c>
       <c r="I21" s="27">
         <f>SUM(F21:H21)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L21" s="26"/>
     </row>
@@ -1993,10 +2020,10 @@
         <v>33</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13">
@@ -2027,16 +2054,16 @@
         <v>2</v>
       </c>
       <c r="B10" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>50</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>53</v>
       </c>
       <c r="F10" s="13">
         <v>2</v>
@@ -2069,10 +2096,10 @@
         <v>34</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14">
@@ -2090,13 +2117,13 @@
         <v>35</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F12" s="13">
         <v>1</v>
@@ -2110,19 +2137,19 @@
         <v>5</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>36</v>
+        <v>95</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>57</v>
+        <v>96</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="F13" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="13">
         <v>1</v>
@@ -2287,13 +2314,13 @@
         <v>1</v>
       </c>
       <c r="B9" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="D9" t="s">
         <v>44</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
       </c>
       <c r="E9" s="34"/>
       <c r="F9" s="34">
@@ -2324,13 +2351,13 @@
         <v>2</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="D10" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="E10" s="13"/>
       <c r="F10" s="13">
@@ -2361,16 +2388,16 @@
         <v>3</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F11" s="14">
         <v>1</v>
@@ -2384,13 +2411,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13">
@@ -2405,13 +2432,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="13">
@@ -2580,13 +2607,13 @@
         <v>1</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13">
@@ -2617,16 +2644,16 @@
         <v>2</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F10" s="13">
         <v>3</v>
@@ -2656,13 +2683,13 @@
         <v>3</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14">
@@ -2677,13 +2704,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13">
@@ -2698,16 +2725,16 @@
         <v>5</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D13" s="41" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F13" s="13">
         <v>1</v>
@@ -2907,7 +2934,7 @@
         <v>32</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13">
@@ -2938,13 +2965,13 @@
         <v>2</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E10" s="13"/>
       <c r="F10" s="13">
@@ -2975,16 +3002,16 @@
         <v>3</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C11" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="42" t="s">
         <v>91</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E11" s="42" t="s">
-        <v>96</v>
       </c>
       <c r="F11" s="14">
         <v>2</v>
@@ -2998,13 +3025,13 @@
         <v>4</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13">
@@ -3022,13 +3049,13 @@
         <v>31</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="F13" s="13">
         <v>1</v>
@@ -3132,14 +3159,14 @@
     </row>
     <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" s="46"/>
       <c r="C2" s="46"/>
     </row>
     <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="B3" s="47"/>
       <c r="C3" s="47"/>
@@ -3192,13 +3219,25 @@
       </c>
     </row>
     <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
+      <c r="A9" s="36">
+        <v>1</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>102</v>
+      </c>
       <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>1</v>
+      </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -3217,13 +3256,25 @@
       <c r="W9" s="5"/>
     </row>
     <row r="10" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="6"/>
+      <c r="A10" s="36">
+        <v>2</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>108</v>
+      </c>
       <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1</v>
+      </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -3242,13 +3293,27 @@
       <c r="W10" s="5"/>
     </row>
     <row r="11" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="36"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="A11" s="36">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="14">
+        <v>1</v>
+      </c>
+      <c r="G11" s="14">
+        <v>2</v>
+      </c>
     </row>
     <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="36"/>

</xml_diff>